<commit_message>
Melhorias e continuação no projeto
</commit_message>
<xml_diff>
--- a/Lista de espécies do Cerrado.xlsx
+++ b/Lista de espécies do Cerrado.xlsx
@@ -1,12 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20416"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rogerio.siqueira\Documents\DEMANDAS\Análise do Inventário Florestal Nacional no Bioma Cerrado\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CB2355C-7925-469F-A914-5CDF7B7DB1DB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25200" windowHeight="11655" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Página1" sheetId="1" r:id="rId4"/>
+    <sheet name="Página1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -310,64 +319,64 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor theme="0"/>
-      </patternFill>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -557,21 +566,25 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:C35"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="27.63"/>
-    <col customWidth="1" min="2" max="3" width="33.75"/>
+    <col min="1" max="1" width="30.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="48.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="87.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -582,7 +595,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -593,7 +606,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -604,18 +617,18 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="1" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
@@ -626,18 +639,18 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="1" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>18</v>
       </c>
@@ -648,7 +661,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>21</v>
       </c>
@@ -659,7 +672,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>24</v>
       </c>
@@ -670,7 +683,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>27</v>
       </c>
@@ -681,7 +694,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>30</v>
       </c>
@@ -692,7 +705,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>32</v>
       </c>
@@ -703,7 +716,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>35</v>
       </c>
@@ -714,7 +727,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>38</v>
       </c>
@@ -725,7 +738,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>40</v>
       </c>
@@ -736,7 +749,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>43</v>
       </c>
@@ -747,7 +760,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>46</v>
       </c>
@@ -758,7 +771,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>49</v>
       </c>
@@ -769,7 +782,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>52</v>
       </c>
@@ -780,7 +793,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>55</v>
       </c>
@@ -791,7 +804,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>58</v>
       </c>
@@ -802,7 +815,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>61</v>
       </c>
@@ -813,7 +826,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>64</v>
       </c>
@@ -824,7 +837,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>64</v>
       </c>
@@ -835,7 +848,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>69</v>
       </c>
@@ -846,7 +859,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>72</v>
       </c>
@@ -857,7 +870,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>75</v>
       </c>
@@ -868,7 +881,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>77</v>
       </c>
@@ -879,7 +892,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>80</v>
       </c>
@@ -890,7 +903,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>83</v>
       </c>
@@ -901,7 +914,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
         <v>86</v>
       </c>
@@ -912,7 +925,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>89</v>
       </c>
@@ -923,7 +936,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
         <v>92</v>
       </c>
@@ -934,7 +947,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
         <v>95</v>
       </c>
@@ -945,10 +958,10 @@
         <v>97</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="C35" s="1"/>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
</xml_diff>